<commit_message>
Correct E_cbl_LTS default to match FEM-confirmed cable modulus
input/WP_TF_input_template.xlsx: E_cbl_LTS default changed from 0.1 GPa to
10 GPa. TF_FEM_benchmark_2026 (TFBM_model.txt, material 1, EX=1e10 Pa)
confirms 10 GPa is the real cable structural modulus; 0.1 GPa was already
flagged as suspect by the FEM package's own review doc and, per the
previous commit, made the new transition SCF overshoot the FEM Jacket
peak by +9%. Updates validation findings accordingly.
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Equivalent Young's modulus of the LTS cable stack</t>
+          <t>Equivalent Young's modulus of the LTS cable stack. Corrected from an earlier default of 0.1 GPa: TF_FEM_benchmark_2026 confirmed the real cable structural modulus is ~10 GPa (ANSYS material 1, EX=1e10 Pa) - see validation/TF_FEM_benchmark_2026_findings.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP: local 3D coil draft and outputs folder (superseded by the uploaded base ZIP in the next commit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2473,6 +2473,206 @@
       <c r="E81" t="inlineStr">
         <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_shape_mode</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>0 = analytic bending-free (Princeton D) shape from the current centroid radii only; 1 = iterate the shape under the real 3D field of all n_TF coils (self as an ideal filament + the other n_TF-1 coils by exact Biot-Savart), falling back to mode 0 if it fails to converge</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_n_seg</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Number of points discretizing the half D-shape (before mirroring) for both the shape solver and the field filaments</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_shape_tol</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Relative change in r and z between shape iterations below which mode 1 is considered converged</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_max_iter</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Maximum shape iterations for tf3d_shape_mode = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_nose_ol_factor</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Outer-leg case nose thickness as a fraction of the inner-leg one (outer leg is far from the peak field and is not sized by the WP-TF solver; this only shapes the CAD export). TO BE CONFIRMED with the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_use_arcs</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>1 = build the 3D filament field model on the manufacturable 3-tangent-arc shape (as it would actually be wound); 0 = build it directly on the smooth bending-free shape</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_n_fil_layer</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Filaments per layer used to represent the other n_TF-1 coils (1 = single filament at the layer's mean radius)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>tf3d_export</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>1 = write the CAD offset-curve and shape-detail files</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
max_cable_aspect_ratio (default 2); magnetic pressure from the J x B field of the field model
- scan rejects cells with Cond_w/Cond_h above max_cable_aspect_ratio
  (input files without it: 2); calibration reference WPs likewise
- p_rs (jacket sizing, jacket radial stress, vault) from the field grade 1
  is sized for: calibrated/discrete peak with field_model 1/2, Ampere x
  corr_B_WP with field_model 0 (unchanged there)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -368,14 +368,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="6" min="1" max="1"/>
+    <col width="26" customWidth="1" style="6" min="2" max="2"/>
+    <col width="14" customWidth="1" style="6" min="3" max="3"/>
+    <col width="8" customWidth="1" style="6" min="4" max="4"/>
+    <col width="78" customWidth="1" style="6" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1331,27 +1331,27 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Numerical settings</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>maxdim</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>30</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Maximum number of grades/layers preallocated per candidate design</t>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>WP dimensioning</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>max_cable_aspect_ratio</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Maximum cell aspect ratio Cond_w/Cond_h; wider cells are rejected</t>
         </is>
       </c>
     </row>
@@ -1363,11 +1363,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Increm</t>
+          <t>maxdim</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Scale factor for cable corner radius/turn insulation (e.g. 1.003 for room-temperature dimensions)</t>
+          <t>Maximum number of grades/layers preallocated per candidate design</t>
         </is>
       </c>
     </row>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>n_grades</t>
+          <t>Increm</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Number of field grades used to segment the winding pack (2 or 3 supported)</t>
+          <t>Scale factor for cable corner radius/turn insulation (e.g. 1.003 for room-temperature dimensions)</t>
         </is>
       </c>
     </row>
@@ -1413,20 +1413,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>grade_B_target_2</t>
+          <t>n_grades</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Target field [T] used to place the 2nd grade transition (only used if n_grades=3)</t>
+          <t>Number of field grades used to segment the winding pack (2 or 3 supported)</t>
         </is>
       </c>
     </row>
@@ -1438,11 +1438,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>grade_B_target_3</t>
+          <t>grade_B_target_2</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Target field [T] used to place the last grade transition</t>
+          <t>Target field [T] used to place the 2nd grade transition (only used if n_grades=3)</t>
         </is>
       </c>
     </row>
@@ -1463,20 +1463,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Iop_min</t>
+          <t>grade_B_target_3</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10000</v>
+        <v>6</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Minimum allowed operating current</t>
+          <t>Target field [T] used to place the last grade transition</t>
         </is>
       </c>
     </row>
@@ -1488,11 +1488,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Iop_max</t>
+          <t>Iop_min</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>70000</v>
+        <v>10000</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Maximum allowed operating current</t>
+          <t>Minimum allowed operating current</t>
         </is>
       </c>
     </row>
@@ -1513,20 +1513,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>min_size_CICC</t>
+          <t>Iop_max</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.015</v>
+        <v>70000</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Minimum feasible CICC conductor size</t>
+          <t>Maximum allowed operating current</t>
         </is>
       </c>
     </row>
@@ -1538,11 +1538,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>max_size_CICC</t>
+          <t>min_size_CICC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.06</v>
+        <v>0.015</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Maximum feasible CICC conductor size</t>
+          <t>Minimum feasible CICC conductor size</t>
         </is>
       </c>
     </row>
@@ -1563,11 +1563,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>min_JT</t>
+          <t>max_size_CICC</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.002</v>
+        <v>0.06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Minimum feasible jacket thickness</t>
+          <t>Maximum feasible CICC conductor size</t>
         </is>
       </c>
     </row>
@@ -1588,11 +1588,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>JT_step</t>
+          <t>min_JT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0001</v>
+        <v>0.002</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Increment used while iteratively sizing the jacket thickness (JT)</t>
+          <t>Minimum feasible jacket thickness</t>
         </is>
       </c>
     </row>
@@ -1613,11 +1613,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>DTF_initial</t>
+          <t>JT_step</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.05</v>
+        <v>0.0001</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Initial guess for the case nose thickness (DTF) sizing search</t>
+          <t>Increment used while iteratively sizing the jacket thickness (JT)</t>
         </is>
       </c>
     </row>
@@ -1638,11 +1638,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>DTF_step</t>
+          <t>DTF_initial</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.001</v>
+        <v>0.05</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Increment used while iteratively sizing the case nose thickness (DTF)</t>
+          <t>Initial guess for the case nose thickness (DTF) sizing search</t>
         </is>
       </c>
     </row>
@@ -1663,11 +1663,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>WP_radial_build_max_est</t>
+          <t>DTF_step</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.5</v>
+        <v>0.001</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Rough estimate of the WP's maximum radial build, used only to bound the combinatorial search (see script comments, fix #2)</t>
+          <t>Increment used while iteratively sizing the case nose thickness (DTF)</t>
         </is>
       </c>
     </row>
@@ -1688,20 +1688,20 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>case_wedge_frac_min</t>
+          <t>WP_radial_build_max_est</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Minimum case wedge (lateral) thickness as a fraction of the case width</t>
+          <t>Rough estimate of the WP's maximum radial build, used only to bound the combinatorial search (see script comments, fix #2)</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1713,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>case_wedge_frac_max</t>
+          <t>case_wedge_frac_min</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.3</v>
+        <v>0.05</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Maximum case wedge (lateral) thickness as a fraction of the case width</t>
+          <t>Minimum case wedge (lateral) thickness as a fraction of the case width</t>
         </is>
       </c>
     </row>
@@ -1738,20 +1738,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>lateral_w_step</t>
+          <t>case_wedge_frac_max</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.02</v>
+        <v>0.3</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Step used to scan the case wedge thickness between its min and max</t>
+          <t>Maximum case wedge (lateral) thickness as a fraction of the case width</t>
         </is>
       </c>
     </row>
@@ -1763,70 +1763,70 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>lateral_w_step</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Step used to scan the case wedge thickness between its min and max</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Numerical settings</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>max_sizing_iterations</t>
         </is>
       </c>
-      <c r="C56" t="n">
+      <c r="C57" t="n">
         <v>100000</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>Safety cap on the iterative sizing loops (jacket, DTF) before raising a non-convergence error</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Structural corrections (provisional)</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>SCF_transition_provisional</t>
         </is>
       </c>
-      <c r="C57" s="2" t="n">
+      <c r="C58" s="2" t="n">
         <v>3.15</v>
       </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>PROVISIONAL, single-point calibration: multiplier on the Jacket primary radial stress (Pm+Pb) at layers adjacent to a grade transition, added because a lumped stiffness-network model cannot reproduce the local bending stress a 2D FEM shows there. Calibrated against exactly one benchmark (TF_FEM_benchmark_2026, 100 turns/2 grades/62.3kA): Jacket SINT=979.6 MPa vs an uncorrected model prediction of ~242 MPa membrane stress contribution at that layer. Revisit once more FEM points are available - see validation/TF_FEM_benchmark_2026_findings.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>T_ref</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>293</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -1838,11 +1838,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>T_op</t>
+          <t>T_ref</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4.2</v>
+        <v>293</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
+          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -1863,20 +1863,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>alpha_steel</t>
+          <t>T_op</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1.038e-05</v>
+        <v>4.2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
+          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
         </is>
       </c>
     </row>
@@ -1888,11 +1888,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>alpha_cable</t>
+          <t>alpha_steel</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>5.54e-06</v>
+        <v>1.038e-05</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the cable (homogenized)</t>
+          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>alpha_ins_n</t>
+          <t>alpha_cable</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2.422e-05</v>
+        <v>5.54e-06</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, through the thickness</t>
+          <t>Secant thermal expansion of the cable (homogenized)</t>
         </is>
       </c>
     </row>
@@ -1938,11 +1938,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>alpha_ins_t</t>
+          <t>alpha_ins_n</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>8.65e-06</v>
+        <v>2.422e-05</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
+          <t>Secant thermal expansion of the insulation, through the thickness</t>
         </is>
       </c>
     </row>
@@ -1963,20 +1963,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>E_ins_t</t>
+          <t>alpha_ins_t</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>20</v>
+        <v>8.65e-06</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
+          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
         </is>
       </c>
     </row>
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>G_ins</t>
+          <t>E_ins_t</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Shear modulus of the insulation</t>
+          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
         </is>
       </c>
     </row>
@@ -2013,20 +2013,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>nu_steel</t>
+          <t>G_ins</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.29</v>
+        <v>6</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Poisson ratio of jacket and case steel</t>
+          <t>Shear modulus of the insulation</t>
         </is>
       </c>
     </row>
@@ -2038,11 +2038,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>nu_cable</t>
+          <t>nu_steel</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Poisson ratio of the cable</t>
+          <t>Poisson ratio of jacket and case steel</t>
         </is>
       </c>
     </row>
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>nu_ins_tn</t>
+          <t>nu_cable</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
+          <t>Poisson ratio of the cable</t>
         </is>
       </c>
     </row>
@@ -2088,11 +2088,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>nu_ins_tz</t>
+          <t>nu_ins_tn</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
         </is>
       </c>
     </row>
@@ -2113,20 +2113,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>E_filler</t>
+          <t>nu_ins_tz</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>7</v>
+        <v>0.17</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Young's modulus of the corner filler between rounded turns</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
         </is>
       </c>
     </row>
@@ -2138,20 +2138,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>nu_filler</t>
+          <t>E_filler</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Poisson ratio of the corner filler</t>
+          <t>Young's modulus of the corner filler between rounded turns</t>
         </is>
       </c>
     </row>
@@ -2163,20 +2163,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>alpha_filler</t>
+          <t>nu_filler</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.73e-05</v>
+        <v>0.3</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the corner filler</t>
+          <t>Poisson ratio of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2188,20 +2188,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>wedge_insulation</t>
+          <t>alpha_filler</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.0015</v>
+        <v>1.73e-05</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
+          <t>Secant thermal expansion of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2213,20 +2213,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>mu_case</t>
+          <t>wedge_insulation</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.2</v>
+        <v>0.0015</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Friction coefficient WP (ground insulation) / case</t>
+          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>mu_cable</t>
+          <t>mu_case</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Friction coefficient cable / jacket</t>
+          <t>Friction coefficient WP (ground insulation) / case</t>
         </is>
       </c>
     </row>
@@ -2263,11 +2263,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>mu_flank</t>
+          <t>mu_cable</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
+          <t>Friction coefficient cable / jacket</t>
         </is>
       </c>
     </row>
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>surrogate_n_cable</t>
+          <t>mu_flank</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Minimum number of elements along each straight jacket wall</t>
+          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
         </is>
       </c>
     </row>
@@ -2313,11 +2313,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>surrogate_n_arc</t>
+          <t>surrogate_n_cable</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Elements along each 90 deg jacket fillet (even)</t>
+          <t>Minimum number of elements along each straight jacket wall</t>
         </is>
       </c>
     </row>
@@ -2338,11 +2338,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>surrogate_n_thk</t>
+          <t>surrogate_n_arc</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Elements through the jacket thickness</t>
+          <t>Elements along each 90 deg jacket fillet (even)</t>
         </is>
       </c>
     </row>
@@ -2363,20 +2363,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>surrogate_h_fine</t>
+          <t>surrogate_n_thk</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.003</v>
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+          <t>Elements through the jacket thickness</t>
         </is>
       </c>
     </row>
@@ -2388,132 +2388,132 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>surrogate_h_fine</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="24" customHeight="1" s="6">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
           <t>surrogate_load_sequence</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C82" t="n">
         <v>0</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="24" customHeight="1">
-      <c r="A82" t="inlineStr">
+    <row r="83" ht="24" customHeight="1" s="6">
+      <c r="A83" t="inlineStr">
         <is>
           <t>Mechanical surrogate</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>surrogate_em_steps</t>
         </is>
       </c>
-      <c r="C82" t="n">
+      <c r="C83" t="n">
         <v>4</v>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
         <is>
           <t>Energization steps when surrogate_load_sequence = 1</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="24" customHeight="1">
-      <c r="A83" t="inlineStr">
+    <row r="84" ht="24" customHeight="1" s="6">
+      <c r="A84" t="inlineStr">
         <is>
           <t>Mechanical surrogate</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>surrogate_classify</t>
         </is>
       </c>
-      <c r="C83" t="n">
+      <c r="C84" t="n">
         <v>1</v>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="24" customHeight="1">
-      <c r="A84" t="inlineStr">
+    <row r="85" ht="24" customHeight="1" s="6">
+      <c r="A85" t="inlineStr">
         <is>
           <t>Mechanical surrogate</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>surrogate_contact_tol</t>
         </is>
       </c>
-      <c r="C84" t="n">
+      <c r="C85" t="n">
         <v>0.005</v>
       </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="24" customHeight="1">
-      <c r="A85" t="inlineStr">
+    <row r="86" ht="24" customHeight="1" s="6">
+      <c r="A86" t="inlineStr">
         <is>
           <t>Mechanical surrogate</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>Sm_jacket</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
-        <v>667000000</v>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Pa</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="24" customHeight="1">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Sm_case</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -2526,380 +2526,405 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
+          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="24" customHeight="1" s="6">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Sm_case</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>667000000</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="24" customHeight="1">
-      <c r="A87" s="7" t="inlineStr">
+    <row r="88" ht="24" customHeight="1" s="6">
+      <c r="A88" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B87" s="7" t="inlineStr">
+      <c r="B88" s="8" t="inlineStr">
         <is>
           <t>tf3d_shape_mode</t>
         </is>
       </c>
-      <c r="C87" s="7" t="n">
+      <c r="C88" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="D88" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E87" s="9" t="inlineStr">
+      <c r="E88" s="9" t="inlineStr">
         <is>
           <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="24" customHeight="1">
-      <c r="A88" s="7" t="inlineStr">
+    <row r="89" ht="24" customHeight="1" s="6">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t>tf3d_n_seg</t>
         </is>
       </c>
-      <c r="C88" s="7" t="n">
+      <c r="C89" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E88" s="9" t="inlineStr">
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
         <is>
           <t>Target segments per closed turn; increase to check convergence</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="7" t="inlineStr">
+    <row r="90" ht="24" customHeight="1" s="6">
+      <c r="A90" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>tf3d_shape_tol</t>
         </is>
       </c>
-      <c r="C89" s="7" t="n">
+      <c r="C90" s="8" t="n">
         <v>0.0001</v>
       </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E89" s="9" t="inlineStr">
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
         <is>
           <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="7" t="inlineStr">
+    <row r="91" ht="24" customHeight="1" s="6">
+      <c r="A91" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B90" s="7" t="inlineStr">
+      <c r="B91" s="8" t="inlineStr">
         <is>
           <t>tf3d_max_iter</t>
         </is>
       </c>
-      <c r="C90" s="7" t="n">
+      <c r="C91" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E90" s="9" t="inlineStr">
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
         <is>
           <t>Maximum experimental shape iterations</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="24" customHeight="1">
-      <c r="A91" s="7" t="inlineStr">
+    <row r="92" ht="24" customHeight="1" s="6">
+      <c r="A92" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="B92" s="8" t="inlineStr">
         <is>
           <t>tf3d_shape_relax</t>
         </is>
       </c>
-      <c r="C91" s="7" t="n">
+      <c r="C92" s="8" t="n">
         <v>0.35</v>
       </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E91" s="9" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
         <is>
           <t>Shape update relaxation; mode 1 only</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="24" customHeight="1">
-      <c r="A92" s="7" t="inlineStr">
+    <row r="93" ht="24" customHeight="1" s="6">
+      <c r="A93" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B92" s="7" t="inlineStr">
+      <c r="B93" s="8" t="inlineStr">
         <is>
           <t>tf3d_nose_ol_factor</t>
         </is>
       </c>
-      <c r="C92" s="7" t="n">
+      <c r="C93" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E92" s="9" t="inlineStr">
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
         <is>
           <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="24" customHeight="1">
-      <c r="A93" s="7" t="inlineStr">
+    <row r="94" ht="24" customHeight="1" s="6">
+      <c r="A94" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="B94" s="8" t="inlineStr">
         <is>
           <t>tf3d_use_arcs</t>
         </is>
       </c>
-      <c r="C93" s="7" t="n">
+      <c r="C94" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D94" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E93" s="9" t="inlineStr">
+      <c r="E94" s="9" t="inlineStr">
         <is>
           <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="24" customHeight="1">
-      <c r="A94" s="7" t="inlineStr">
+    <row r="95" ht="24" customHeight="1" s="6">
+      <c r="A95" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B94" s="7" t="inlineStr">
+      <c r="B95" s="8" t="inlineStr">
         <is>
           <t>tf3d_export</t>
         </is>
       </c>
-      <c r="C94" s="7" t="n">
+      <c r="C95" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="D95" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E94" s="9" t="inlineStr">
+      <c r="E95" s="9" t="inlineStr">
         <is>
           <t>Export CAD curves after numerical and geometric checks</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="24" customHeight="1">
-      <c r="A95" s="7" t="inlineStr">
+    <row r="96" ht="24" customHeight="1" s="6">
+      <c r="A96" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B95" s="7" t="inlineStr">
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t>tf3d_neighbor_gauss</t>
         </is>
       </c>
-      <c r="C95" s="7" t="n">
+      <c r="C96" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D95" s="7" t="inlineStr">
+      <c r="D96" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E95" s="9" t="inlineStr">
+      <c r="E96" s="9" t="inlineStr">
         <is>
           <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="24" customHeight="1">
-      <c r="A96" s="7" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="B97" s="8" t="inlineStr">
         <is>
           <t>tf3d_source_block</t>
         </is>
       </c>
-      <c r="C96" s="7" t="n">
+      <c r="C97" s="8" t="n">
         <v>512</v>
       </c>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E96" s="9" t="inlineStr">
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="inlineStr">
         <is>
           <t>Maximum source segments per field evaluation block</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="7" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="B98" s="8" t="inlineStr">
         <is>
           <t>tf3d_point_block</t>
         </is>
       </c>
-      <c r="C97" s="7" t="n">
+      <c r="C98" s="8" t="n">
         <v>128</v>
       </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E97" s="9" t="inlineStr">
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
         <is>
           <t>Maximum field points per block</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="7" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B98" s="7" t="inlineStr">
+      <c r="B99" s="8" t="inlineStr">
         <is>
           <t>tf3d_n_eval</t>
         </is>
       </c>
-      <c r="C98" s="7" t="n">
+      <c r="C99" s="8" t="n">
         <v>48</v>
       </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E98" s="9" t="inlineStr">
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="inlineStr">
         <is>
           <t>Upper-half field/force sample bins; refine for force convergence</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="7" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B99" s="7" t="inlineStr">
+      <c r="B100" s="8" t="inlineStr">
         <is>
           <t>tf3d_arc_tol</t>
         </is>
       </c>
-      <c r="C99" s="7" t="n">
+      <c r="C100" s="8" t="n">
         <v>0.01</v>
       </c>
-      <c r="D99" s="7" t="inlineStr">
+      <c r="D100" s="8" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E99" s="9" t="inlineStr">
+      <c r="E100" s="9" t="inlineStr">
         <is>
           <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="7" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B100" s="7" t="inlineStr">
+      <c r="B101" s="8" t="inlineStr">
         <is>
           <t>tf3d_ampere_tol</t>
         </is>
       </c>
-      <c r="C100" s="7" t="n">
+      <c r="C101" s="8" t="n">
         <v>0.001</v>
       </c>
-      <c r="D100" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E100" s="9" t="inlineStr">
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E101" s="9" t="inlineStr">
         <is>
           <t>Relative tolerance on numerically averaged Ampere field</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="7" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
         <is>
           <t>3D coil</t>
         </is>
       </c>
-      <c r="B101" s="7" t="inlineStr">
+      <c r="B102" s="8" t="inlineStr">
         <is>
           <t>tf3d_energy</t>
         </is>
       </c>
-      <c r="C101" s="7" t="n">
+      <c r="C102" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D101" s="7" t="inlineStr">
+      <c r="D102" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E101" s="9" t="inlineStr">
+      <c r="E102" s="9" t="inlineStr">
         <is>
           <t>0 = off; 1 = approximate centroid-loop energy, no sizing feedback</t>
         </is>
@@ -2919,7 +2944,7 @@
   <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" style="6" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2929,9 +2954,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
WIP jacket stress surrogate option (scf_model, default 0 = unchanged)
- scan: scf_model 1 checks jacket primary Pm / Pm+Pb per layer from
  JACKET_STRESS_SURROGATE against Sm / 1.5 Sm (as the FE figure of merit);
  the nose is then sized by the vault criteria only; RIS refused
- size_case_vault: optional jacket_in_loop, returns S_z
- input template: scf_model; new DATA columns JT_Pm, JT_PmPb
- jacket_stress_surrogate is a placeholder that errors until calibrated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="6" min="1" max="1"/>
@@ -1826,32 +1826,32 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>PROVISIONAL, single-point calibration: multiplier on the Jacket primary radial stress (Pm+Pb) at layers adjacent to a grade transition, added because a lumped stiffness-network model cannot reproduce the local bending stress a 2D FEM shows there. Calibrated against exactly one benchmark (TF_FEM_benchmark_2026, 100 turns/2 grades/62.3kA): Jacket SINT=979.6 MPa vs an uncorrected model prediction of ~242 MPa membrane stress contribution at that layer. Revisit once more FEM points are available - see validation/TF_FEM_benchmark_2026_findings.md.</t>
+          <t>Used with scf_model = 0 only. PROVISIONAL, single-point calibration: multiplier on the Jacket primary radial stress (Pm+Pb) at layers adjacent to a grade transition, added because a lumped stiffness-network model cannot reproduce the local bending stress a 2D FEM shows there. Calibrated against exactly one benchmark (TF_FEM_benchmark_2026, 100 turns/2 grades/62.3kA): Jacket SINT=979.6 MPa vs an uncorrected model prediction of ~242 MPa membrane stress contribution at that layer. Revisit once more FEM points are available - see validation/TF_FEM_benchmark_2026_findings.md.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>T_ref</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>293</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Reference (stress-free) temperature for the cool-down load</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>scf_model</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Jacket stress in the scan: 0 = analytic formula with the SCF table and SCF_transition_provisional (default); 1 = fast surrogate calibrated on the 2D FE: primary Pm and Pm+Pb per layer checked as the FE figure of merit (Pm &lt;= Sm_jacket, Pm+Pb &lt;= 1.5 Sm_jacket), rectangular cables only</t>
         </is>
       </c>
     </row>
@@ -1863,11 +1863,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>T_op</t>
+          <t>T_ref</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4.2</v>
+        <v>293</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
+          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -1888,20 +1888,20 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>alpha_steel</t>
+          <t>T_op</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.038e-05</v>
+        <v>4.2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
+          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
         </is>
       </c>
     </row>
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>alpha_cable</t>
+          <t>alpha_steel</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5.54e-06</v>
+        <v>1.038e-05</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the cable (homogenized)</t>
+          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -1938,11 +1938,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>alpha_ins_n</t>
+          <t>alpha_cable</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2.422e-05</v>
+        <v>5.54e-06</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, through the thickness</t>
+          <t>Secant thermal expansion of the cable (homogenized)</t>
         </is>
       </c>
     </row>
@@ -1963,11 +1963,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>alpha_ins_t</t>
+          <t>alpha_ins_n</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8.65e-06</v>
+        <v>2.422e-05</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
+          <t>Secant thermal expansion of the insulation, through the thickness</t>
         </is>
       </c>
     </row>
@@ -1988,20 +1988,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>E_ins_t</t>
+          <t>alpha_ins_t</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>20</v>
+        <v>8.65e-06</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
+          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
         </is>
       </c>
     </row>
@@ -2013,11 +2013,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>G_ins</t>
+          <t>E_ins_t</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Shear modulus of the insulation</t>
+          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
         </is>
       </c>
     </row>
@@ -2038,20 +2038,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>nu_steel</t>
+          <t>G_ins</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.29</v>
+        <v>6</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Poisson ratio of jacket and case steel</t>
+          <t>Shear modulus of the insulation</t>
         </is>
       </c>
     </row>
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>nu_cable</t>
+          <t>nu_steel</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Poisson ratio of the cable</t>
+          <t>Poisson ratio of jacket and case steel</t>
         </is>
       </c>
     </row>
@@ -2088,11 +2088,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>nu_ins_tn</t>
+          <t>nu_cable</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
+          <t>Poisson ratio of the cable</t>
         </is>
       </c>
     </row>
@@ -2113,11 +2113,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>nu_ins_tz</t>
+          <t>nu_ins_tn</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
         </is>
       </c>
     </row>
@@ -2138,20 +2138,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>E_filler</t>
+          <t>nu_ins_tz</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>7</v>
+        <v>0.17</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Young's modulus of the corner filler between rounded turns</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
         </is>
       </c>
     </row>
@@ -2163,20 +2163,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>nu_filler</t>
+          <t>E_filler</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Poisson ratio of the corner filler</t>
+          <t>Young's modulus of the corner filler between rounded turns</t>
         </is>
       </c>
     </row>
@@ -2188,20 +2188,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>alpha_filler</t>
+          <t>nu_filler</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.73e-05</v>
+        <v>0.3</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the corner filler</t>
+          <t>Poisson ratio of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2213,20 +2213,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>wedge_insulation</t>
+          <t>alpha_filler</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.0015</v>
+        <v>1.73e-05</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
+          <t>Secant thermal expansion of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2238,20 +2238,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>mu_case</t>
+          <t>wedge_insulation</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.2</v>
+        <v>0.0015</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Friction coefficient WP (ground insulation) / case</t>
+          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>mu_cable</t>
+          <t>mu_case</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Friction coefficient cable / jacket</t>
+          <t>Friction coefficient WP (ground insulation) / case</t>
         </is>
       </c>
     </row>
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>mu_flank</t>
+          <t>mu_cable</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
+          <t>Friction coefficient cable / jacket</t>
         </is>
       </c>
     </row>
@@ -2313,11 +2313,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>surrogate_n_cable</t>
+          <t>mu_flank</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Minimum number of elements along each straight jacket wall</t>
+          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
         </is>
       </c>
     </row>
@@ -2338,11 +2338,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>surrogate_n_arc</t>
+          <t>surrogate_n_cable</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Elements along each 90 deg jacket fillet (even)</t>
+          <t>Minimum number of elements along each straight jacket wall</t>
         </is>
       </c>
     </row>
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>surrogate_n_thk</t>
+          <t>surrogate_n_arc</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Elements through the jacket thickness</t>
+          <t>Elements along each 90 deg jacket fillet (even)</t>
         </is>
       </c>
     </row>
@@ -2388,20 +2388,20 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>surrogate_h_fine</t>
+          <t>surrogate_n_thk</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.003</v>
+        <v>2</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+          <t>Elements through the jacket thickness</t>
         </is>
       </c>
     </row>
@@ -2413,20 +2413,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>surrogate_load_sequence</t>
+          <t>surrogate_h_fine</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
+          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
         </is>
       </c>
     </row>
@@ -2438,20 +2438,20 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>surrogate_em_steps</t>
+          <t>surrogate_load_sequence</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Energization steps when surrogate_load_sequence = 1</t>
+          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
         </is>
       </c>
     </row>
@@ -2463,11 +2463,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>surrogate_classify</t>
+          <t>surrogate_em_steps</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+          <t>Energization steps when surrogate_load_sequence = 1</t>
         </is>
       </c>
     </row>
@@ -2488,11 +2488,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>surrogate_contact_tol</t>
+          <t>surrogate_classify</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.005</v>
+        <v>1</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
         </is>
       </c>
     </row>
@@ -2513,20 +2513,20 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Sm_jacket</t>
+          <t>surrogate_contact_tol</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>667000000</v>
+        <v>0.005</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Sm_case</t>
+          <t>Sm_jacket</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -2551,32 +2551,32 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
+          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="24" customHeight="1" s="6">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sm_case</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>667000000</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="24" customHeight="1" s="6">
-      <c r="A88" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B88" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_mode</t>
-        </is>
-      </c>
-      <c r="C88" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D88" s="8" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E88" s="9" t="inlineStr">
-        <is>
-          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2588,20 +2588,20 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_seg</t>
+          <t>tf3d_shape_mode</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>Target segments per closed turn; increase to check convergence</t>
+          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2613,11 +2613,11 @@
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_tol</t>
+          <t>tf3d_n_seg</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>0.0001</v>
+        <v>180</v>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Unrelaxed shape update / radial span; mode 1 only</t>
+          <t>Target segments per closed turn; increase to check convergence</t>
         </is>
       </c>
     </row>
@@ -2638,11 +2638,11 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>tf3d_max_iter</t>
+          <t>tf3d_shape_tol</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>20</v>
+        <v>0.0001</v>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Maximum experimental shape iterations</t>
+          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2663,11 +2663,11 @@
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_relax</t>
+          <t>tf3d_max_iter</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>0.35</v>
+        <v>20</v>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Shape update relaxation; mode 1 only</t>
+          <t>Maximum experimental shape iterations</t>
         </is>
       </c>
     </row>
@@ -2688,11 +2688,11 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>tf3d_nose_ol_factor</t>
+          <t>tf3d_shape_relax</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
+          <t>Shape update relaxation; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2713,20 +2713,20 @@
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>tf3d_use_arcs</t>
+          <t>tf3d_nose_ol_factor</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
+          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
         </is>
       </c>
     </row>
@@ -2738,11 +2738,11 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>tf3d_export</t>
+          <t>tf3d_use_arcs</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>Export CAD curves after numerical and geometric checks</t>
+          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
         </is>
       </c>
     </row>
@@ -2763,11 +2763,11 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>tf3d_neighbor_gauss</t>
+          <t>tf3d_export</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
+          <t>Export CAD curves after numerical and geometric checks</t>
         </is>
       </c>
     </row>
@@ -2788,20 +2788,20 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>tf3d_source_block</t>
+          <t>tf3d_neighbor_gauss</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>512</v>
+        <v>2</v>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Maximum source segments per field evaluation block</t>
+          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
         </is>
       </c>
     </row>
@@ -2813,11 +2813,11 @@
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>tf3d_point_block</t>
+          <t>tf3d_source_block</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>128</v>
+        <v>512</v>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Maximum field points per block</t>
+          <t>Maximum source segments per field evaluation block</t>
         </is>
       </c>
     </row>
@@ -2838,11 +2838,11 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_eval</t>
+          <t>tf3d_point_block</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Upper-half field/force sample bins; refine for force convergence</t>
+          <t>Maximum field points per block</t>
         </is>
       </c>
     </row>
@@ -2863,20 +2863,20 @@
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>tf3d_arc_tol</t>
+          <t>tf3d_n_eval</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>0.01</v>
+        <v>48</v>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+          <t>Upper-half field/force sample bins; refine for force convergence</t>
         </is>
       </c>
     </row>
@@ -2888,20 +2888,20 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>tf3d_ampere_tol</t>
+          <t>tf3d_arc_tol</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Relative tolerance on numerically averaged Ampere field</t>
+          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
         </is>
       </c>
     </row>
@@ -2913,18 +2913,43 @@
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
+          <t>tf3d_ampere_tol</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>Relative tolerance on numerically averaged Ampere field</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
           <t>tf3d_energy</t>
         </is>
       </c>
-      <c r="C102" s="8" t="n">
+      <c r="C103" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D102" s="8" t="inlineStr">
+      <c r="D103" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E102" s="9" t="inlineStr">
+      <c r="E103" s="9" t="inlineStr">
         <is>
           <t>0 = off; 1 = approximate centroid-loop energy, no sizing feedback</t>
         </is>
@@ -2954,7 +2979,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
MADE-2.0: jacket surrogate recalibrated with jacket-thickness variants; JT sized per grade in the scan
- 12 FE runs of thicker-jacket variants of 6 base designs added to the
  calibration (2 excluded: WP out of the sector); new form with
  (JT/3mm)^0.2 and a width-step term, coefficients refitted
- scf_model = 1 sizes JT per grade (jacket_margin 1.10, JT_max,
  jacket_max_passes in the input template), results ranked by radial build
- jacket_jt_variant returns the minimum toroidal gap
- docs/DIMENSIONAMENTO_JACKET.md: calibration results and sizing method

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="6" min="1" max="1"/>
@@ -1851,82 +1851,82 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Jacket stress in the scan: 0 = analytic formula with the SCF table and SCF_transition_provisional (default); 1 = fast surrogate calibrated on the 2D FE: primary Pm and Pm+Pb per layer checked as the FE figure of merit (Pm &lt;= Sm_jacket, Pm+Pb &lt;= 1.5 Sm_jacket), rectangular cables only</t>
+          <t>Jacket stress in the scan: 0 = analytic formula with the SCF table and SCF_transition_provisional (default); 1 = fast surrogate calibrated on the 2D FE (jacket_stress_surrogate): the jacket thickness of every grade is SIZED (smallest JT with jacket_margin x Pm &lt;= Sm_jacket and jacket_margin x Pm+Pb &lt;= 1.5 Sm_jacket), iterated with the case nose; rectangular cables only. See docs/DIMENSIONAMENTO_JACKET.md</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>T_ref</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>293</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Reference (stress-free) temperature for the cool-down load</t>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>jacket_margin</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Used with scf_model = 1: factor on the surrogate jacket stresses when sizing JT. Surrogate vs 2D FE on the design maximum Pm+Pb (leave-one-design-out, 23 runs): median 1.03, 80th percentile 1.13, max 1.23. 1.10 covers about 75% of the calibration designs; the chosen design is verified with the 2D FE</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>T_op</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>JT_max</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Used with scf_model = 1: largest jacket thickness the sizing may reach; a candidate that needs more is rejected</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>alpha_steel</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>1.038e-05</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>1/K</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>jacket_max_passes</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Used with scf_model = 1: maximum number of extra sizing passes of a candidate when its jacket grows (WP height, stiffness and axial stress change)</t>
         </is>
       </c>
     </row>
@@ -1938,20 +1938,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>alpha_cable</t>
+          <t>T_ref</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>5.54e-06</v>
+        <v>293</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the cable (homogenized)</t>
+          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -1963,20 +1963,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>alpha_ins_n</t>
+          <t>T_op</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2.422e-05</v>
+        <v>4.2</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, through the thickness</t>
+          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
         </is>
       </c>
     </row>
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>alpha_ins_t</t>
+          <t>alpha_steel</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>8.65e-06</v>
+        <v>1.038e-05</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
+          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -2013,20 +2013,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>E_ins_t</t>
+          <t>alpha_cable</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>20</v>
+        <v>5.54e-06</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
+          <t>Secant thermal expansion of the cable (homogenized)</t>
         </is>
       </c>
     </row>
@@ -2038,20 +2038,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>G_ins</t>
+          <t>alpha_ins_n</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6</v>
+        <v>2.422e-05</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Shear modulus of the insulation</t>
+          <t>Secant thermal expansion of the insulation, through the thickness</t>
         </is>
       </c>
     </row>
@@ -2063,20 +2063,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>nu_steel</t>
+          <t>alpha_ins_t</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.29</v>
+        <v>8.65e-06</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Poisson ratio of jacket and case steel</t>
+          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
         </is>
       </c>
     </row>
@@ -2088,20 +2088,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>nu_cable</t>
+          <t>E_ins_t</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.3</v>
+        <v>20</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Poisson ratio of the cable</t>
+          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
         </is>
       </c>
     </row>
@@ -2113,20 +2113,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>nu_ins_tn</t>
+          <t>G_ins</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.33</v>
+        <v>6</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
+          <t>Shear modulus of the insulation</t>
         </is>
       </c>
     </row>
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>nu_ins_tz</t>
+          <t>nu_steel</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.17</v>
+        <v>0.29</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
+          <t>Poisson ratio of jacket and case steel</t>
         </is>
       </c>
     </row>
@@ -2163,20 +2163,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>E_filler</t>
+          <t>nu_cable</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>7</v>
+        <v>0.3</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Young's modulus of the corner filler between rounded turns</t>
+          <t>Poisson ratio of the cable</t>
         </is>
       </c>
     </row>
@@ -2188,11 +2188,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>nu_filler</t>
+          <t>nu_ins_tn</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Poisson ratio of the corner filler</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
         </is>
       </c>
     </row>
@@ -2213,20 +2213,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>alpha_filler</t>
+          <t>nu_ins_tz</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.73e-05</v>
+        <v>0.17</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the corner filler</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
         </is>
       </c>
     </row>
@@ -2238,20 +2238,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>wedge_insulation</t>
+          <t>E_filler</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.0015</v>
+        <v>7</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
+          <t>Young's modulus of the corner filler between rounded turns</t>
         </is>
       </c>
     </row>
@@ -2263,11 +2263,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>mu_case</t>
+          <t>nu_filler</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Friction coefficient WP (ground insulation) / case</t>
+          <t>Poisson ratio of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2288,20 +2288,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>mu_cable</t>
+          <t>alpha_filler</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.2</v>
+        <v>1.73e-05</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Friction coefficient cable / jacket</t>
+          <t>Secant thermal expansion of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2313,20 +2313,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>mu_flank</t>
+          <t>wedge_insulation</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>0.0015</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
+          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
         </is>
       </c>
     </row>
@@ -2338,11 +2338,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>surrogate_n_cable</t>
+          <t>mu_case</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>0.2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Minimum number of elements along each straight jacket wall</t>
+          <t>Friction coefficient WP (ground insulation) / case</t>
         </is>
       </c>
     </row>
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>surrogate_n_arc</t>
+          <t>mu_cable</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>8</v>
+        <v>0.2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Elements along each 90 deg jacket fillet (even)</t>
+          <t>Friction coefficient cable / jacket</t>
         </is>
       </c>
     </row>
@@ -2388,11 +2388,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>surrogate_n_thk</t>
+          <t>mu_flank</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Elements through the jacket thickness</t>
+          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
         </is>
       </c>
     </row>
@@ -2413,20 +2413,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>surrogate_h_fine</t>
+          <t>surrogate_n_cable</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.003</v>
+        <v>4</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+          <t>Minimum number of elements along each straight jacket wall</t>
         </is>
       </c>
     </row>
@@ -2438,20 +2438,20 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>surrogate_load_sequence</t>
+          <t>surrogate_n_arc</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
+          <t>Elements along each 90 deg jacket fillet (even)</t>
         </is>
       </c>
     </row>
@@ -2463,11 +2463,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>surrogate_em_steps</t>
+          <t>surrogate_n_thk</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Energization steps when surrogate_load_sequence = 1</t>
+          <t>Elements through the jacket thickness</t>
         </is>
       </c>
     </row>
@@ -2488,20 +2488,20 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>surrogate_classify</t>
+          <t>surrogate_h_fine</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>0.003</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
         </is>
       </c>
     </row>
@@ -2513,20 +2513,20 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>surrogate_contact_tol</t>
+          <t>surrogate_load_sequence</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
         </is>
       </c>
     </row>
@@ -2538,20 +2538,20 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Sm_jacket</t>
+          <t>surrogate_em_steps</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>667000000</v>
+        <v>4</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+          <t>Energization steps when surrogate_load_sequence = 1</t>
         </is>
       </c>
     </row>
@@ -2563,95 +2563,95 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
+          <t>surrogate_classify</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="24" customHeight="1" s="6">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>surrogate_contact_tol</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="24" customHeight="1" s="6">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Sm_jacket</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>667000000</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="24" customHeight="1" s="6">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>Sm_case</t>
         </is>
       </c>
-      <c r="C88" t="n">
+      <c r="C91" t="n">
         <v>667000000</v>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="24" customHeight="1" s="6">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B89" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_mode</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D89" s="8" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E89" s="9" t="inlineStr">
-        <is>
-          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="24" customHeight="1" s="6">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_n_seg</t>
-        </is>
-      </c>
-      <c r="C90" s="8" t="n">
-        <v>180</v>
-      </c>
-      <c r="D90" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E90" s="9" t="inlineStr">
-        <is>
-          <t>Target segments per closed turn; increase to check convergence</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="24" customHeight="1" s="6">
-      <c r="A91" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_tol</t>
-        </is>
-      </c>
-      <c r="C91" s="8" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D91" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E91" s="9" t="inlineStr">
-        <is>
-          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2663,20 +2663,20 @@
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>tf3d_max_iter</t>
+          <t>tf3d_shape_mode</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Maximum experimental shape iterations</t>
+          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2688,11 +2688,11 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_relax</t>
+          <t>tf3d_n_seg</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>0.35</v>
+        <v>180</v>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E93" s="9" t="inlineStr">
         <is>
-          <t>Shape update relaxation; mode 1 only</t>
+          <t>Target segments per closed turn; increase to check convergence</t>
         </is>
       </c>
     </row>
@@ -2713,11 +2713,11 @@
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>tf3d_nose_ol_factor</t>
+          <t>tf3d_shape_tol</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>0.5</v>
+        <v>0.0001</v>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
+          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2738,20 +2738,20 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>tf3d_use_arcs</t>
+          <t>tf3d_max_iter</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr">
         <is>
-          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
+          <t>Maximum experimental shape iterations</t>
         </is>
       </c>
     </row>
@@ -2763,20 +2763,20 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>tf3d_export</t>
+          <t>tf3d_shape_relax</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Export CAD curves after numerical and geometric checks</t>
+          <t>Shape update relaxation; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2788,20 +2788,20 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>tf3d_neighbor_gauss</t>
+          <t>tf3d_nose_ol_factor</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
+          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
         </is>
       </c>
     </row>
@@ -2813,20 +2813,20 @@
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>tf3d_source_block</t>
+          <t>tf3d_use_arcs</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>512</v>
+        <v>0</v>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Maximum source segments per field evaluation block</t>
+          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
         </is>
       </c>
     </row>
@@ -2838,20 +2838,20 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>tf3d_point_block</t>
+          <t>tf3d_export</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>128</v>
+        <v>1</v>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Maximum field points per block</t>
+          <t>Export CAD curves after numerical and geometric checks</t>
         </is>
       </c>
     </row>
@@ -2863,20 +2863,20 @@
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_eval</t>
+          <t>tf3d_neighbor_gauss</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Upper-half field/force sample bins; refine for force convergence</t>
+          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
         </is>
       </c>
     </row>
@@ -2888,20 +2888,20 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>tf3d_arc_tol</t>
+          <t>tf3d_source_block</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>0.01</v>
+        <v>512</v>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+          <t>Maximum source segments per field evaluation block</t>
         </is>
       </c>
     </row>
@@ -2913,11 +2913,11 @@
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>tf3d_ampere_tol</t>
+          <t>tf3d_point_block</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>0.001</v>
+        <v>128</v>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Relative tolerance on numerically averaged Ampere field</t>
+          <t>Maximum field points per block</t>
         </is>
       </c>
     </row>
@@ -2938,18 +2938,93 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
+          <t>tf3d_n_eval</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="inlineStr">
+        <is>
+          <t>Upper-half field/force sample bins; refine for force convergence</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>tf3d_arc_tol</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D104" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="inlineStr">
+        <is>
+          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>tf3d_ampere_tol</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>Relative tolerance on numerically averaged Ampere field</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
           <t>tf3d_energy</t>
         </is>
       </c>
-      <c r="C103" s="8" t="n">
+      <c r="C106" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D103" s="8" t="inlineStr">
+      <c r="D106" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E103" s="9" t="inlineStr">
+      <c r="E106" s="9" t="inlineStr">
         <is>
           <t>0 = off; 1 = approximate centroid-loop energy, no sizing feedback</t>
         </is>

</xml_diff>

<commit_message>
MADE-2.0: jacket sizing with the FE-calibrated surrogate (scf_model = 1) is the default
The analytic formula (scf_model = 0) with SCF_transition_provisional rejects
every wide winding pack with 3 grades (diagnostic scan: only W 304-344 mm
pass), while the surrogate keeps the wide ones. RIS cables fall back to
scf_model = 0 with a warning instead of stopping the scan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Jacket stress in the scan: 0 = analytic formula with the SCF table and SCF_transition_provisional (default); 1 = fast surrogate calibrated on the 2D FE (jacket_stress_surrogate): the jacket thickness of every grade is SIZED (smallest JT with jacket_margin x Pm &lt;= Sm_jacket and jacket_margin x Pm+Pb &lt;= 1.5 Sm_jacket), iterated with the case nose; rectangular cables only. See docs/DIMENSIONAMENTO_JACKET.md</t>
+          <t>Jacket stress in the scan: 1 = fast surrogate calibrated on the 2D FE (jacket_stress_surrogate, default): the jacket thickness of every grade is SIZED (smallest JT with jacket_margin x Pm &lt;= Sm_jacket and jacket_margin x Pm+Pb &lt;= 1.5 Sm_jacket), iterated with the case nose; rectangular cables (RIS falls back to 0). 0 = analytic formula with the SCF table and SCF_transition_provisional: it under-predicts the FE by up to 62% and penalizes wide cells, so with 3 grades it keeps only narrow winding packs. See docs/DIMENSIONAMENTO_JACKET.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tau_delay from the input file: fixed value or ITER criterion
Input template: Tau_delay_mode (0 fixed, 1 ITER), Tau_delay, v_quench_LTS.
ITER mode: dump 2 s after the normal zone reaches 0.1 V (ITER TF quench
analysis assumptions), detection time from QUENCH_DELAY_TIME; HTS grades
keep the fixed value. cicc_params(p) applies the input overrides; scan,
field calibration and the hot-spot plot use the same delay per grade.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016ZB4vBvf3mBq51RYw47c7s
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="6" min="1" max="1"/>
@@ -1106,102 +1106,102 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Electrical</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>V_MAX</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>2500</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Maximum allowed voltage during a fast discharge</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Thermal allowables</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Tau_delay_mode</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Quench delay before the dump: 0 = fixed value Tau_delay; 1 = ITER criterion (time to reach the 0.1 V detection voltage + 2 s, see conductor/quench_delay_time.m; HTS keeps Tau_delay)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>WP dimensioning</t>
+          <t>Thermal allowables</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>toroidal_gap</t>
+          <t>Tau_delay</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.015</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>s</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Minimum required toroidal gap between WP and case at every grade</t>
+          <t>Fixed quench delay (Tau_delay_mode = 0, and HTS grades with Tau_delay_mode = 1)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>WP dimensioning</t>
+          <t>Thermal allowables</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>GoundIns</t>
+          <t>v_quench_LTS</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.005</v>
+        <v>5</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ground insulation thickness around the winding pack</t>
+          <t>Normal-zone propagation speed in the LTS CICC (Tau_delay_mode = 1 only)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>WP dimensioning</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>INS_grades</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Insulation thickness between adjacent WP grades</t>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>V_MAX</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Maximum allowed voltage during a fast discharge</t>
         </is>
       </c>
     </row>
@@ -1213,11 +1213,11 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>turn_insulation_nominal</t>
+          <t>toroidal_gap</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.001</v>
+        <v>0.015</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Nominal turn insulation thickness per face (scaled by Increm)</t>
+          <t>Minimum required toroidal gap between WP and case at every grade</t>
         </is>
       </c>
     </row>
@@ -1238,11 +1238,11 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>r_SC_min</t>
+          <t>GoundIns</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Minimum cable corner fillet radius</t>
+          <t>Ground insulation thickness around the winding pack</t>
         </is>
       </c>
     </row>
@@ -1263,11 +1263,11 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>r_SC_max</t>
+          <t>INS_grades</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.006</v>
+        <v>0.0005</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Maximum cable corner fillet radius. General rule (not a free input): r_SC = JT, clamped to [r_SC_min, r_SC_max] - the fillet tracks the jacket thickness up to this cap, then stays fixed.</t>
+          <t>Insulation thickness between adjacent WP grades</t>
         </is>
       </c>
     </row>
@@ -1288,11 +1288,11 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>min_SC_w</t>
+          <t>turn_insulation_nominal</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Minimum feasible superconductor cable width (geometric feasibility floor)</t>
+          <t>Nominal turn insulation thickness per face (scaled by Increm)</t>
         </is>
       </c>
     </row>
@@ -1313,20 +1313,20 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>min_cable_aspect_ratio</t>
+          <t>r_SC_min</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.99</v>
+        <v>0.002</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Minimum acceptable Cond_w/Cond_h cable aspect ratio</t>
+          <t>Minimum cable corner fillet radius</t>
         </is>
       </c>
     </row>
@@ -1338,95 +1338,95 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>r_SC_max</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Maximum cable corner fillet radius. General rule (not a free input): r_SC = JT, clamped to [r_SC_min, r_SC_max] - the fillet tracks the jacket thickness up to this cap, then stays fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>WP dimensioning</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>min_SC_w</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Minimum feasible superconductor cable width (geometric feasibility floor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>WP dimensioning</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>min_cable_aspect_ratio</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Minimum acceptable Cond_w/Cond_h cable aspect ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>WP dimensioning</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
           <t>max_cable_aspect_ratio</t>
         </is>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C42" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Maximum cell aspect ratio Cond_w/Cond_h; wider cells are rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Numerical settings</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>maxdim</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>30</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Maximum number of grades/layers preallocated per candidate design</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Numerical settings</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Increm</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Scale factor for cable corner radius/turn insulation (e.g. 1.003 for room-temperature dimensions)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Numerical settings</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>n_grades</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>3</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Number of field grades used to segment the winding pack (2 or 3 supported)</t>
         </is>
       </c>
     </row>
@@ -1438,20 +1438,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>grade_B_target_2</t>
+          <t>maxdim</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Target field [T] used to place the 2nd grade transition (only used if n_grades=3)</t>
+          <t>Maximum number of grades/layers preallocated per candidate design</t>
         </is>
       </c>
     </row>
@@ -1463,20 +1463,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>grade_B_target_3</t>
+          <t>Increm</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Target field [T] used to place the last grade transition</t>
+          <t>Scale factor for cable corner radius/turn insulation (e.g. 1.003 for room-temperature dimensions)</t>
         </is>
       </c>
     </row>
@@ -1488,20 +1488,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Iop_min</t>
+          <t>n_grades</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>10000</v>
+        <v>3</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Minimum allowed operating current</t>
+          <t>Number of field grades used to segment the winding pack (2 or 3 supported)</t>
         </is>
       </c>
     </row>
@@ -1513,20 +1513,20 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Iop_max</t>
+          <t>grade_B_target_2</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>70000</v>
+        <v>9</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Maximum allowed operating current</t>
+          <t>Target field [T] used to place the 2nd grade transition (only used if n_grades=3)</t>
         </is>
       </c>
     </row>
@@ -1538,20 +1538,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>min_size_CICC</t>
+          <t>grade_B_target_3</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.015</v>
+        <v>6</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Minimum feasible CICC conductor size</t>
+          <t>Target field [T] used to place the last grade transition</t>
         </is>
       </c>
     </row>
@@ -1563,20 +1563,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>max_size_CICC</t>
+          <t>Iop_min</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.06</v>
+        <v>10000</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Maximum feasible CICC conductor size</t>
+          <t>Minimum allowed operating current</t>
         </is>
       </c>
     </row>
@@ -1588,20 +1588,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>min_JT</t>
+          <t>Iop_max</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.002</v>
+        <v>70000</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Minimum feasible jacket thickness</t>
+          <t>Maximum allowed operating current</t>
         </is>
       </c>
     </row>
@@ -1613,11 +1613,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>JT_step</t>
+          <t>min_size_CICC</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.0001</v>
+        <v>0.015</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Increment used while iteratively sizing the jacket thickness (JT)</t>
+          <t>Minimum feasible CICC conductor size</t>
         </is>
       </c>
     </row>
@@ -1638,11 +1638,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>DTF_initial</t>
+          <t>max_size_CICC</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Initial guess for the case nose thickness (DTF) sizing search</t>
+          <t>Maximum feasible CICC conductor size</t>
         </is>
       </c>
     </row>
@@ -1663,11 +1663,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>DTF_step</t>
+          <t>min_JT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Increment used while iteratively sizing the case nose thickness (DTF)</t>
+          <t>Minimum feasible jacket thickness</t>
         </is>
       </c>
     </row>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WP_radial_build_max_est</t>
+          <t>JT_step</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.5</v>
+        <v>0.0001</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Rough estimate of the WP's maximum radial build, used only to bound the combinatorial search (see script comments, fix #2)</t>
+          <t>Increment used while iteratively sizing the jacket thickness (JT)</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>case_wedge_frac_min</t>
+          <t>DTF_initial</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1721,12 +1721,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Minimum case wedge (lateral) thickness as a fraction of the case width</t>
+          <t>Initial guess for the case nose thickness (DTF) sizing search</t>
         </is>
       </c>
     </row>
@@ -1738,20 +1738,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>case_wedge_frac_max</t>
+          <t>DTF_step</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.3</v>
+        <v>0.001</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Maximum case wedge (lateral) thickness as a fraction of the case width</t>
+          <t>Increment used while iteratively sizing the case nose thickness (DTF)</t>
         </is>
       </c>
     </row>
@@ -1763,11 +1763,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>lateral_w_step</t>
+          <t>WP_radial_build_max_est</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.02</v>
+        <v>0.5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Step used to scan the case wedge thickness between its min and max</t>
+          <t>Rough estimate of the WP's maximum radial build, used only to bound the combinatorial search (see script comments, fix #2)</t>
         </is>
       </c>
     </row>
@@ -1788,95 +1788,95 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>case_wedge_frac_min</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Minimum case wedge (lateral) thickness as a fraction of the case width</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Numerical settings</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>case_wedge_frac_max</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Maximum case wedge (lateral) thickness as a fraction of the case width</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Numerical settings</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>lateral_w_step</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Step used to scan the case wedge thickness between its min and max</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Numerical settings</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>max_sizing_iterations</t>
         </is>
       </c>
-      <c r="C57" t="n">
+      <c r="C60" t="n">
         <v>100000</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>Safety cap on the iterative sizing loops (jacket, DTF) before raising a non-convergence error</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Structural corrections (provisional)</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>SCF_transition_provisional</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Used with scf_model = 0 only. PROVISIONAL, single-point calibration: multiplier on the Jacket primary radial stress (Pm+Pb) at layers adjacent to a grade transition, added because a lumped stiffness-network model cannot reproduce the local bending stress a 2D FEM shows there. Calibrated against exactly one benchmark (TF_FEM_benchmark_2026, 100 turns/2 grades/62.3kA): Jacket SINT=979.6 MPa vs an uncorrected model prediction of ~242 MPa membrane stress contribution at that layer. Revisit once more FEM points are available - see validation/TF_FEM_benchmark_2026_findings.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Structural corrections (provisional)</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>scf_model</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Jacket stress in the scan: 1 = fast surrogate calibrated on the 2D FE (jacket_stress_surrogate, default): the jacket thickness of every grade is SIZED (smallest JT with jacket_margin x Pm &lt;= Sm_jacket and jacket_margin x Pm+Pb &lt;= 1.5 Sm_jacket), iterated with the case nose; rectangular cables (RIS falls back to 0). 0 = analytic formula with the SCF table and SCF_transition_provisional: it under-predicts the FE by up to 62% and penalizes wide cells, so with 3 grades it keeps only narrow winding packs. See docs/DIMENSIONAMENTO_JACKET.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Structural corrections (provisional)</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>jacket_margin</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Used with scf_model = 1: factor on the surrogate jacket stresses when sizing JT. Surrogate vs 2D FE on the design maximum Pm+Pb (leave-one-design-out, 23 runs): median 1.03, 80th percentile 1.13, max 1.23. 1.10 covers about 75% of the calibration designs; the chosen design is verified with the 2D FE</t>
         </is>
       </c>
     </row>
@@ -1888,20 +1888,20 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>JT_max</t>
+          <t>SCF_transition_provisional</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>0.01</v>
+        <v>3.15</v>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Used with scf_model = 1: largest jacket thickness the sizing may reach; a candidate that needs more is rejected</t>
+          <t>Used with scf_model = 0 only. PROVISIONAL, single-point calibration: multiplier on the Jacket primary radial stress (Pm+Pb) at layers adjacent to a grade transition, added because a lumped stiffness-network model cannot reproduce the local bending stress a 2D FEM shows there. Calibrated against exactly one benchmark (TF_FEM_benchmark_2026, 100 turns/2 grades/62.3kA): Jacket SINT=979.6 MPa vs an uncorrected model prediction of ~242 MPa membrane stress contribution at that layer. Revisit once more FEM points are available - see validation/TF_FEM_benchmark_2026_findings.md.</t>
         </is>
       </c>
     </row>
@@ -1913,20 +1913,20 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>jacket_max_passes</t>
+          <t>scf_model</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Used with scf_model = 1: maximum number of extra sizing passes of a candidate when its jacket grows (WP height, stiffness and axial stress change)</t>
+          <t>Jacket stress in the scan: 1 = fast surrogate calibrated on the 2D FE (jacket_stress_surrogate, default): the jacket thickness of every grade is SIZED (smallest JT with jacket_margin x Pm &lt;= Sm_jacket and jacket_margin x Pm+Pb &lt;= 1.5 Sm_jacket), iterated with the case nose; rectangular cables (RIS falls back to 0). 0 = analytic formula with the SCF table and SCF_transition_provisional: it under-predicts the FE by up to 62% and penalizes wide cells, so with 3 grades it keeps only narrow winding packs. See docs/DIMENSIONAMENTO_JACKET.md</t>
         </is>
       </c>
     </row>
@@ -1938,20 +1938,20 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>case_model</t>
+          <t>jacket_margin</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>1 = case nose sized with the case stress surrogate calibrated on the 2D FE (layered model x g(h_WP/t_nose), max case Pm and Pm+Pb vs Sm_case; docs/MODELLO_A_STRATI.md section 11); 0 = analytic vault formula</t>
+          <t>Used with scf_model = 1: factor on the surrogate jacket stresses when sizing JT. Surrogate vs 2D FE on the design maximum Pm+Pb (leave-one-design-out, 23 runs): median 1.03, 80th percentile 1.13, max 1.23. 1.10 covers about 75% of the calibration designs; the chosen design is verified with the 2D FE</t>
         </is>
       </c>
     </row>
@@ -1963,20 +1963,20 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>case_margin</t>
+          <t>JT_max</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>1.05</v>
+        <v>0.01</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Used with case_model = 1: factor on the surrogate case Pm when sizing the nose. Leave-one-design-out vs 2D FE (19 runs): model/FE 0.967-1.040, rms 2.1%</t>
+          <t>Used with scf_model = 1: largest jacket thickness the sizing may reach; a candidate that needs more is rejected</t>
         </is>
       </c>
     </row>
@@ -1988,95 +1988,95 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
+          <t>jacket_max_passes</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Used with scf_model = 1: maximum number of extra sizing passes of a candidate when its jacket grows (WP height, stiffness and axial stress change)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>case_model</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>1 = case nose sized with the case stress surrogate calibrated on the 2D FE (layered model x g(h_WP/t_nose), max case Pm and Pm+Pb vs Sm_case; docs/MODELLO_A_STRATI.md section 11); 0 = analytic vault formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>case_margin</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Used with case_model = 1: factor on the surrogate case Pm when sizing the nose. Leave-one-design-out vs 2D FE (19 runs): model/FE 0.967-1.040, rms 2.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
           <t>case_margin_PmPb</t>
         </is>
       </c>
-      <c r="C65" s="2" t="n">
+      <c r="C68" s="2" t="n">
         <v>1.1</v>
       </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>Used with case_model = 1: factor on the surrogate case Pm+Pb. Leave-one-design-out vs 2D FE: model/FE 0.864-1.121, rms 7.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>T_ref</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>293</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Reference (stress-free) temperature for the cool-down load</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>T_op</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>alpha_steel</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>1.038e-05</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>1/K</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -2088,20 +2088,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>alpha_cable</t>
+          <t>T_ref</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5.54e-06</v>
+        <v>293</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the cable (homogenized)</t>
+          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -2113,20 +2113,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>alpha_ins_n</t>
+          <t>T_op</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2.422e-05</v>
+        <v>4.2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, through the thickness</t>
+          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
         </is>
       </c>
     </row>
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>alpha_ins_t</t>
+          <t>alpha_steel</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>8.65e-06</v>
+        <v>1.038e-05</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
+          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -2163,20 +2163,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>E_ins_t</t>
+          <t>alpha_cable</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>20</v>
+        <v>5.54e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
+          <t>Secant thermal expansion of the cable (homogenized)</t>
         </is>
       </c>
     </row>
@@ -2188,20 +2188,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>G_ins</t>
+          <t>alpha_ins_n</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>2.422e-05</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Shear modulus of the insulation</t>
+          <t>Secant thermal expansion of the insulation, through the thickness</t>
         </is>
       </c>
     </row>
@@ -2213,20 +2213,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>nu_steel</t>
+          <t>alpha_ins_t</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.29</v>
+        <v>8.65e-06</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Poisson ratio of jacket and case steel</t>
+          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
         </is>
       </c>
     </row>
@@ -2238,20 +2238,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>nu_cable</t>
+          <t>E_ins_t</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.3</v>
+        <v>20</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Poisson ratio of the cable</t>
+          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
         </is>
       </c>
     </row>
@@ -2263,20 +2263,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>nu_ins_tn</t>
+          <t>G_ins</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.33</v>
+        <v>6</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
+          <t>Shear modulus of the insulation</t>
         </is>
       </c>
     </row>
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>nu_ins_tz</t>
+          <t>nu_steel</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.17</v>
+        <v>0.29</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
+          <t>Poisson ratio of jacket and case steel</t>
         </is>
       </c>
     </row>
@@ -2313,20 +2313,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>E_filler</t>
+          <t>nu_cable</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>0.3</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Young's modulus of the corner filler between rounded turns</t>
+          <t>Poisson ratio of the cable</t>
         </is>
       </c>
     </row>
@@ -2338,11 +2338,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>nu_filler</t>
+          <t>nu_ins_tn</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Poisson ratio of the corner filler</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
         </is>
       </c>
     </row>
@@ -2363,20 +2363,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>alpha_filler</t>
+          <t>nu_ins_tz</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.73e-05</v>
+        <v>0.17</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the corner filler</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
         </is>
       </c>
     </row>
@@ -2388,20 +2388,20 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>wedge_insulation</t>
+          <t>E_filler</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.0015</v>
+        <v>7</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
+          <t>Young's modulus of the corner filler between rounded turns</t>
         </is>
       </c>
     </row>
@@ -2413,11 +2413,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>mu_case</t>
+          <t>nu_filler</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Friction coefficient WP (ground insulation) / case</t>
+          <t>Poisson ratio of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2438,20 +2438,20 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>mu_cable</t>
+          <t>alpha_filler</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.2</v>
+        <v>1.73e-05</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Friction coefficient cable / jacket</t>
+          <t>Secant thermal expansion of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2463,20 +2463,20 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>mu_flank</t>
+          <t>wedge_insulation</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0</v>
+        <v>0.0015</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
+          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
         </is>
       </c>
     </row>
@@ -2488,11 +2488,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>surrogate_n_cable</t>
+          <t>mu_case</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>0.2</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Minimum number of elements along each straight jacket wall</t>
+          <t>Friction coefficient WP (ground insulation) / case</t>
         </is>
       </c>
     </row>
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>surrogate_n_arc</t>
+          <t>mu_cable</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>0.2</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Elements along each 90 deg jacket fillet (even)</t>
+          <t>Friction coefficient cable / jacket</t>
         </is>
       </c>
     </row>
@@ -2538,11 +2538,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>surrogate_n_thk</t>
+          <t>mu_flank</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Elements through the jacket thickness</t>
+          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
         </is>
       </c>
     </row>
@@ -2563,20 +2563,20 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>surrogate_h_fine</t>
+          <t>surrogate_n_cable</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.003</v>
+        <v>4</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+          <t>Minimum number of elements along each straight jacket wall</t>
         </is>
       </c>
     </row>
@@ -2588,20 +2588,20 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>surrogate_load_sequence</t>
+          <t>surrogate_n_arc</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
+          <t>Elements along each 90 deg jacket fillet (even)</t>
         </is>
       </c>
     </row>
@@ -2613,11 +2613,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>surrogate_em_steps</t>
+          <t>surrogate_n_thk</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Energization steps when surrogate_load_sequence = 1</t>
+          <t>Elements through the jacket thickness</t>
         </is>
       </c>
     </row>
@@ -2638,20 +2638,20 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>surrogate_classify</t>
+          <t>surrogate_h_fine</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>0.003</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
         </is>
       </c>
     </row>
@@ -2663,20 +2663,20 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>surrogate_contact_tol</t>
+          <t>surrogate_load_sequence</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
         </is>
       </c>
     </row>
@@ -2688,20 +2688,20 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Sm_jacket</t>
+          <t>surrogate_em_steps</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>667000000</v>
+        <v>4</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+          <t>Energization steps when surrogate_load_sequence = 1</t>
         </is>
       </c>
     </row>
@@ -2713,95 +2713,95 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
+          <t>surrogate_classify</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="24" customHeight="1" s="6">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>surrogate_contact_tol</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="24" customHeight="1" s="6">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Sm_jacket</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>667000000</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
           <t>Sm_case</t>
         </is>
       </c>
-      <c r="C94" t="n">
+      <c r="C97" t="n">
         <v>667000000</v>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D97" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E97" t="inlineStr">
         <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="24" customHeight="1" s="6">
-      <c r="A95" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_mode</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E95" s="9" t="inlineStr">
-        <is>
-          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="24" customHeight="1" s="6">
-      <c r="A96" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B96" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_n_seg</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="n">
-        <v>180</v>
-      </c>
-      <c r="D96" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E96" s="9" t="inlineStr">
-        <is>
-          <t>Target segments per closed turn; increase to check convergence</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B97" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_tol</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D97" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E97" s="9" t="inlineStr">
-        <is>
-          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2813,20 +2813,20 @@
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>tf3d_max_iter</t>
+          <t>tf3d_shape_mode</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Maximum experimental shape iterations</t>
+          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2838,11 +2838,11 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_relax</t>
+          <t>tf3d_n_seg</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>0.35</v>
+        <v>180</v>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Shape update relaxation; mode 1 only</t>
+          <t>Target segments per closed turn; increase to check convergence</t>
         </is>
       </c>
     </row>
@@ -2863,11 +2863,11 @@
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>tf3d_nose_ol_factor</t>
+          <t>tf3d_shape_tol</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>0.5</v>
+        <v>0.0001</v>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
+          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2888,20 +2888,20 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>tf3d_use_arcs</t>
+          <t>tf3d_max_iter</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
+          <t>Maximum experimental shape iterations</t>
         </is>
       </c>
     </row>
@@ -2913,20 +2913,20 @@
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>tf3d_export</t>
+          <t>tf3d_shape_relax</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Export CAD curves after numerical and geometric checks</t>
+          <t>Shape update relaxation; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2938,20 +2938,20 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>tf3d_neighbor_gauss</t>
+          <t>tf3d_nose_ol_factor</t>
         </is>
       </c>
       <c r="C103" s="8" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
+          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
         </is>
       </c>
     </row>
@@ -2963,20 +2963,20 @@
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>tf3d_source_block</t>
+          <t>tf3d_use_arcs</t>
         </is>
       </c>
       <c r="C104" s="8" t="n">
-        <v>512</v>
+        <v>0</v>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Maximum source segments per field evaluation block</t>
+          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
         </is>
       </c>
     </row>
@@ -2988,20 +2988,20 @@
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>tf3d_point_block</t>
+          <t>tf3d_export</t>
         </is>
       </c>
       <c r="C105" s="8" t="n">
-        <v>128</v>
+        <v>1</v>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Maximum field points per block</t>
+          <t>Export CAD curves after numerical and geometric checks</t>
         </is>
       </c>
     </row>
@@ -3013,20 +3013,20 @@
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_eval</t>
+          <t>tf3d_neighbor_gauss</t>
         </is>
       </c>
       <c r="C106" s="8" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Upper-half field/force sample bins; refine for force convergence</t>
+          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
         </is>
       </c>
     </row>
@@ -3038,20 +3038,20 @@
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>tf3d_arc_tol</t>
+          <t>tf3d_source_block</t>
         </is>
       </c>
       <c r="C107" s="8" t="n">
-        <v>0.01</v>
+        <v>512</v>
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+          <t>Maximum source segments per field evaluation block</t>
         </is>
       </c>
     </row>
@@ -3063,11 +3063,11 @@
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>tf3d_ampere_tol</t>
+          <t>tf3d_point_block</t>
         </is>
       </c>
       <c r="C108" s="8" t="n">
-        <v>0.001</v>
+        <v>128</v>
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Relative tolerance on numerically averaged Ampere field</t>
+          <t>Maximum field points per block</t>
         </is>
       </c>
     </row>
@@ -3088,18 +3088,93 @@
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
+          <t>tf3d_n_eval</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="D109" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>Upper-half field/force sample bins; refine for force convergence</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>tf3d_arc_tol</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D110" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>tf3d_ampere_tol</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D111" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Relative tolerance on numerically averaged Ampere field</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
           <t>tf3d_energy</t>
         </is>
       </c>
-      <c r="C109" s="8" t="n">
+      <c r="C112" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D109" s="8" t="inlineStr">
+      <c r="D112" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E109" s="9" t="inlineStr">
+      <c r="E112" s="9" t="inlineStr">
         <is>
           <t>0 = off; 1 = approximate centroid-loop energy, no sizing feedback</t>
         </is>

</xml_diff>

<commit_message>
Coupled sizing with the 3D beam + shell global model, linked to the main run
- tf3d_global_from_design: global model (STR_360 counterpart) built from the
  chosen design: centroid line, 3D Lorentz forces of all coils, case + jacket
  beam section (tf3d_section_from_design), vault shells from the design
- axial_load_factor: inner-leg vertical force / T_bf, applied to T_bf in the
  scan, size_case_vault, layered model, surrogates, 2D FE, refine_jacket_fe,
  ANSYS export (AXIAL_LOAD_FACTOR read by Solution_STR.f)
- resize_design_point: re-sizes one candidate (scan stores n_turns0; scan
  options cal/quiet); couple_global_sizing iterates sizing <-> global model
- main step 6b: global model, coupled sizing, FE check; plot_tf3d_global
- template: axial_load_factor and g3d_* parameters

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VoSJvBN9muunahFTxoAR2X
</commit_message>
<xml_diff>
--- a/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
+++ b/MADE-2.0/matlab/input/WP_TF_input_template.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="6" min="1" max="1"/>
@@ -2006,27 +2006,27 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Mechanical surrogate</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>T_ref</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>293</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Reference (stress-free) temperature for the cool-down load</t>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Structural corrections (provisional)</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>axial_load_factor</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Vertical force of the inner leg / bending-free T_bf = 0.5 k_bf n_TF (N I)^2 mu0/(2 pi), used by every sizing and verification step (scan, layered model, case and jacket surrogates, 2D FE, ANSYS export). 1 = formula (half of the vertical force of the upper half). The 3D beam + shell global model of the chosen design gives the real value (main step 6b, coupled sizing); set it here to scan the machine with it</t>
         </is>
       </c>
     </row>
@@ -2038,11 +2038,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>T_op</t>
+          <t>T_ref</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4.2</v>
+        <v>293</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
+          <t>Reference (stress-free) temperature for the cool-down load</t>
         </is>
       </c>
     </row>
@@ -2063,20 +2063,20 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>alpha_steel</t>
+          <t>T_op</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1.038e-05</v>
+        <v>4.2</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
+          <t>Operating temperature (cool-down T_ref -&gt; T_op)</t>
         </is>
       </c>
     </row>
@@ -2088,11 +2088,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>alpha_cable</t>
+          <t>alpha_steel</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5.54e-06</v>
+        <v>1.038e-05</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the cable (homogenized)</t>
+          <t>Secant thermal expansion of jacket and case steel, T_ref -&gt; T_op</t>
         </is>
       </c>
     </row>
@@ -2113,11 +2113,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>alpha_ins_n</t>
+          <t>alpha_cable</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2.422e-05</v>
+        <v>5.54e-06</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, through the thickness</t>
+          <t>Secant thermal expansion of the cable (homogenized)</t>
         </is>
       </c>
     </row>
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>alpha_ins_t</t>
+          <t>alpha_ins_n</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>8.65e-06</v>
+        <v>2.422e-05</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
+          <t>Secant thermal expansion of the insulation, through the thickness</t>
         </is>
       </c>
     </row>
@@ -2163,20 +2163,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>E_ins_t</t>
+          <t>alpha_ins_t</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>20</v>
+        <v>8.65e-06</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
+          <t>Secant thermal expansion of the insulation, in-plane and axial</t>
         </is>
       </c>
     </row>
@@ -2188,11 +2188,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>G_ins</t>
+          <t>E_ins_t</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Shear modulus of the insulation</t>
+          <t>Young's modulus of the insulation, in-plane and axial (E_ins is the through-thickness one)</t>
         </is>
       </c>
     </row>
@@ -2213,20 +2213,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>nu_steel</t>
+          <t>G_ins</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0.29</v>
+        <v>6</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Poisson ratio of jacket and case steel</t>
+          <t>Shear modulus of the insulation</t>
         </is>
       </c>
     </row>
@@ -2238,11 +2238,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>nu_cable</t>
+          <t>nu_steel</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Poisson ratio of the cable</t>
+          <t>Poisson ratio of jacket and case steel</t>
         </is>
       </c>
     </row>
@@ -2263,11 +2263,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>nu_ins_tn</t>
+          <t>nu_cable</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
+          <t>Poisson ratio of the cable</t>
         </is>
       </c>
     </row>
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>nu_ins_tz</t>
+          <t>nu_ins_tn</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.17</v>
+        <v>0.33</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; through-thickness, major)</t>
         </is>
       </c>
     </row>
@@ -2313,20 +2313,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>E_filler</t>
+          <t>nu_ins_tz</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>0.17</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>GPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Young's modulus of the corner filler between rounded turns</t>
+          <t>Insulation Poisson ratio (in-plane -&gt; axial)</t>
         </is>
       </c>
     </row>
@@ -2338,20 +2338,20 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>nu_filler</t>
+          <t>E_filler</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.3</v>
+        <v>7</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>GPa</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Poisson ratio of the corner filler</t>
+          <t>Young's modulus of the corner filler between rounded turns</t>
         </is>
       </c>
     </row>
@@ -2363,20 +2363,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>alpha_filler</t>
+          <t>nu_filler</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.73e-05</v>
+        <v>0.3</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1/K</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Secant thermal expansion of the corner filler</t>
+          <t>Poisson ratio of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2388,20 +2388,20 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>wedge_insulation</t>
+          <t>alpha_filler</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.0015</v>
+        <v>1.73e-05</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>1/K</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
+          <t>Secant thermal expansion of the corner filler</t>
         </is>
       </c>
     </row>
@@ -2413,20 +2413,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>mu_case</t>
+          <t>wedge_insulation</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.2</v>
+        <v>0.0015</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Friction coefficient WP (ground insulation) / case</t>
+          <t>Insulation thickness on the case flanks (wedged inner leg)</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>mu_cable</t>
+          <t>mu_case</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Friction coefficient cable / jacket</t>
+          <t>Friction coefficient WP (ground insulation) / case</t>
         </is>
       </c>
     </row>
@@ -2463,11 +2463,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>mu_flank</t>
+          <t>mu_cable</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
+          <t>Friction coefficient cable / jacket</t>
         </is>
       </c>
     </row>
@@ -2488,11 +2488,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>surrogate_n_cable</t>
+          <t>mu_flank</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Minimum number of elements along each straight jacket wall</t>
+          <t>Friction on the case flanks. 0 as in the FEM: the wedge insulation is constrained only normally on its outer face, so it slides with the case and the case/insulation friction carries no load</t>
         </is>
       </c>
     </row>
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>surrogate_n_arc</t>
+          <t>surrogate_n_cable</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Elements along each 90 deg jacket fillet (even)</t>
+          <t>Minimum number of elements along each straight jacket wall</t>
         </is>
       </c>
     </row>
@@ -2538,11 +2538,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>surrogate_n_thk</t>
+          <t>surrogate_n_arc</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Elements through the jacket thickness</t>
+          <t>Elements along each 90 deg jacket fillet (even)</t>
         </is>
       </c>
     </row>
@@ -2563,20 +2563,20 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>surrogate_h_fine</t>
+          <t>surrogate_n_thk</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.003</v>
+        <v>2</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
+          <t>Elements through the jacket thickness</t>
         </is>
       </c>
     </row>
@@ -2588,20 +2588,20 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>surrogate_load_sequence</t>
+          <t>surrogate_h_fine</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
+          <t>Element size of the case/ground-insulation mesh near the WP and the case boundary</t>
         </is>
       </c>
     </row>
@@ -2613,20 +2613,20 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>surrogate_em_steps</t>
+          <t>surrogate_load_sequence</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Energization steps when surrogate_load_sequence = 1</t>
+          <t>0 = cool-down, Lorentz and axial load applied together in one step (as the ANSYS runs used for validation); 1 = cool-down first, then energization in surrogate_em_steps steps (friction is path dependent)</t>
         </is>
       </c>
     </row>
@@ -2638,11 +2638,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>surrogate_classify</t>
+          <t>surrogate_em_steps</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
+          <t>Energization steps when surrogate_load_sequence = 1</t>
         </is>
       </c>
     </row>
@@ -2663,11 +2663,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>surrogate_contact_tol</t>
+          <t>surrogate_classify</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.005</v>
+        <v>1</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
+          <t>1 = also solve the primary load case (Lorentz + axial, no cool-down) and classify P / P+Q; 0 = total stresses used as primary (conservative, half the run time)</t>
         </is>
       </c>
     </row>
@@ -2688,20 +2688,20 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Sm_jacket</t>
+          <t>surrogate_contact_tol</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>667000000</v>
+        <v>0.005</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+          <t>Contact iterations stop when at most this fraction of the contact pairs still change state; otherwise the result is flagged invalid</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Sm_case</t>
+          <t>Sm_jacket</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2726,32 +2726,32 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
+          <t>Design stress intensity Sm of the jacket steel at the operating temperature used by the stress criteria (Pm &lt;= Sm, Pm+Pb &lt;= 1.5 Sm, P+Q &lt;= 3 Sm). TO BE CONFIRMED against the design code/material data; default = S_amm_JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="24" customHeight="1" s="6">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Mechanical surrogate</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Sm_case</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>667000000</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Pa</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
           <t>Design stress intensity Sm of the case steel (same criteria). TO BE CONFIRMED; default = S_amm_VT</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="24" customHeight="1" s="6">
-      <c r="A95" s="8" t="inlineStr">
-        <is>
-          <t>3D coil</t>
-        </is>
-      </c>
-      <c r="B95" s="8" t="inlineStr">
-        <is>
-          <t>tf3d_shape_mode</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E95" s="9" t="inlineStr">
-        <is>
-          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2763,20 +2763,20 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_seg</t>
+          <t>tf3d_shape_mode</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E96" s="9" t="inlineStr">
         <is>
-          <t>Target segments per closed turn; increase to check convergence</t>
+          <t>0 = analytic Princeton D; 1 = experimental 3D field iteration</t>
         </is>
       </c>
     </row>
@@ -2788,11 +2788,11 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_tol</t>
+          <t>tf3d_n_seg</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>0.0001</v>
+        <v>180</v>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="E97" s="9" t="inlineStr">
         <is>
-          <t>Unrelaxed shape update / radial span; mode 1 only</t>
+          <t>Target segments per closed turn; increase to check convergence</t>
         </is>
       </c>
     </row>
@@ -2813,11 +2813,11 @@
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>tf3d_max_iter</t>
+          <t>tf3d_shape_tol</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>20</v>
+        <v>0.0001</v>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
-          <t>Maximum experimental shape iterations</t>
+          <t>Unrelaxed shape update / radial span; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2838,11 +2838,11 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>tf3d_shape_relax</t>
+          <t>tf3d_max_iter</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>0.35</v>
+        <v>20</v>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E99" s="9" t="inlineStr">
         <is>
-          <t>Shape update relaxation; mode 1 only</t>
+          <t>Maximum experimental shape iterations</t>
         </is>
       </c>
     </row>
@@ -2863,11 +2863,11 @@
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>tf3d_nose_ol_factor</t>
+          <t>tf3d_shape_relax</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E100" s="9" t="inlineStr">
         <is>
-          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
+          <t>Shape update relaxation; mode 1 only</t>
         </is>
       </c>
     </row>
@@ -2888,20 +2888,20 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>tf3d_use_arcs</t>
+          <t>tf3d_nose_ol_factor</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E101" s="9" t="inlineStr">
         <is>
-          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
+          <t>Assumed outer-leg / inner-leg nose thickness ratio</t>
         </is>
       </c>
     </row>
@@ -2913,11 +2913,11 @@
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>tf3d_export</t>
+          <t>tf3d_use_arcs</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>Export CAD curves after numerical and geometric checks</t>
+          <t>0 = free-span geometry; 1 = three-arc fit, subject to arc tolerance</t>
         </is>
       </c>
     </row>
@@ -2938,11 +2938,11 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>tf3d_neighbor_gauss</t>
+          <t>tf3d_export</t>
         </is>
       </c>
       <c r="C103" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="E103" s="9" t="inlineStr">
         <is>
-          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
+          <t>Export CAD curves after numerical and geometric checks</t>
         </is>
       </c>
     </row>
@@ -2963,20 +2963,20 @@
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>tf3d_source_block</t>
+          <t>tf3d_neighbor_gauss</t>
         </is>
       </c>
       <c r="C104" s="8" t="n">
-        <v>512</v>
+        <v>2</v>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
-          <t>Maximum source segments per field evaluation block</t>
+          <t>0 = all turns; 1 or 2 = sources per neighbour-coil layer</t>
         </is>
       </c>
     </row>
@@ -2988,11 +2988,11 @@
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>tf3d_point_block</t>
+          <t>tf3d_source_block</t>
         </is>
       </c>
       <c r="C105" s="8" t="n">
-        <v>128</v>
+        <v>512</v>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>Maximum field points per block</t>
+          <t>Maximum source segments per field evaluation block</t>
         </is>
       </c>
     </row>
@@ -3013,11 +3013,11 @@
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>tf3d_n_eval</t>
+          <t>tf3d_point_block</t>
         </is>
       </c>
       <c r="C106" s="8" t="n">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="E106" s="9" t="inlineStr">
         <is>
-          <t>Upper-half field/force sample bins; refine for force convergence</t>
+          <t>Maximum field points per block</t>
         </is>
       </c>
     </row>
@@ -3038,20 +3038,20 @@
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>tf3d_arc_tol</t>
+          <t>tf3d_n_eval</t>
         </is>
       </c>
       <c r="C107" s="8" t="n">
-        <v>0.01</v>
+        <v>48</v>
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
+          <t>Upper-half field/force sample bins; refine for force convergence</t>
         </is>
       </c>
     </row>
@@ -3063,20 +3063,20 @@
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>tf3d_ampere_tol</t>
+          <t>tf3d_arc_tol</t>
         </is>
       </c>
       <c r="C108" s="8" t="n">
-        <v>0.001</v>
+        <v>0.01</v>
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Relative tolerance on numerically averaged Ampere field</t>
+          <t>Maximum bidirectional fit deviation; blocks arc-based export</t>
         </is>
       </c>
     </row>
@@ -3088,20 +3088,145 @@
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
+          <t>tf3d_ampere_tol</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D109" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>Relative tolerance on numerically averaged Ampere field</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>3D coil</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
           <t>tf3d_energy</t>
         </is>
       </c>
-      <c r="C109" s="8" t="n">
+      <c r="C110" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D109" s="8" t="inlineStr">
+      <c r="D110" s="8" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E109" s="9" t="inlineStr">
+      <c r="E110" s="9" t="inlineStr">
         <is>
           <t>0 = off; 1 = approximate centroid-loop energy, no sizing feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>3D global model</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>g3d_n_seg</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="D111" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Beam elements per coil along the current centroid line (STR_360: 161)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>3D global model</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>g3d_n_gauss</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D112" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>Gauss filaments per direction of the WP section for the 3D Lorentz forces (as MAG_360 SOURC36 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>3D global model</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>g3d_t_ois</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D113" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>Thickness of the outer intercoil structure shells (STR_360: 0.14 m); the vault shells take the steel crossing the coil mid plane (nose + plate + jacket walls) from the design</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>3D global model</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>g3d_axial_mode</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="8" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>Axial load factor from the global model: 0 = inner-leg vertical force (beam + vault shells); 1 = extreme fibre, adds the in-plane bending of the inner leg</t>
         </is>
       </c>
     </row>

</xml_diff>